<commit_message>
[update] Mouse mode is updated.
</commit_message>
<xml_diff>
--- a/misc/keymap.xlsx
+++ b/misc/keymap.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1208" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1159" uniqueCount="215">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -418,6 +418,24 @@
   </si>
   <si>
     <t xml:space="preserve">A+F11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">マウスモード</t>
+  </si>
+  <si>
+    <t xml:space="preserve">左クリック</t>
+  </si>
+  <si>
+    <t xml:space="preserve">右クリック</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WhlUp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WhlDn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Back</t>
   </si>
   <si>
     <t xml:space="preserve">標準(レジストリ編集)</t>
@@ -658,7 +676,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="游ゴシック"/>
@@ -697,6 +715,12 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="7"/>
       <name val="游ゴシック"/>
       <family val="3"/>
       <charset val="128"/>
@@ -926,6 +950,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -934,7 +962,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -952,10 +980,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2439,51 +2463,23 @@
       <c r="O2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="Q2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="R2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="T2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="U2" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="W2" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="X2" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="Y2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="Z2" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="AA2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="AE2" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="Q2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="2"/>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2"/>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
+      <c r="AE2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
@@ -2529,48 +2525,26 @@
         <v>19</v>
       </c>
       <c r="O3" s="2"/>
-      <c r="Q3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Z3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="AB3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="AC3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="AD3" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z3" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2615,45 +2589,27 @@
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
-      <c r="Q4" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="R4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="U4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="V4" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="2"/>
       <c r="W4" s="2" t="s">
-        <v>26</v>
+        <v>135</v>
       </c>
       <c r="X4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y4" s="2" t="s">
-        <v>28</v>
+        <v>53</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="Z4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="AA4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="AB4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC4" s="2" t="s">
-        <v>32</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
       <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
     </row>
@@ -2699,45 +2655,23 @@
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
-      <c r="Q5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="R5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="S5" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="T5" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="U5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="V5" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="W5" s="3" t="s">
-        <v>39</v>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="2" t="s">
+        <v>136</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="Z5" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="AA5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="AB5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="AC5" s="2" t="s">
-        <v>33</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3"/>
+      <c r="AB5" s="3"/>
+      <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
     </row>
@@ -2777,39 +2711,19 @@
       </c>
       <c r="N6" s="6"/>
       <c r="O6" s="6"/>
-      <c r="Q6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="R6" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="S6" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="T6" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="U6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="V6" s="3" t="s">
-        <v>49</v>
-      </c>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
       <c r="W6" s="3"/>
-      <c r="X6" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="Y6" s="3" t="s">
-        <v>58</v>
-      </c>
+      <c r="X6" s="3"/>
+      <c r="Y6" s="3"/>
       <c r="Z6" s="6"/>
-      <c r="AA6" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="AA6" s="2"/>
       <c r="AB6" s="6"/>
-      <c r="AC6" s="2" t="s">
-        <v>52</v>
-      </c>
+      <c r="AC6" s="2"/>
       <c r="AD6" s="6"/>
       <c r="AE6" s="6"/>
     </row>
@@ -2846,37 +2760,31 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="6"/>
       <c r="AA7" s="2"/>
-      <c r="AB7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="AD7" s="2" t="s">
-        <v>55</v>
-      </c>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2893,7 +2801,7 @@
       <c r="N9" s="12"/>
       <c r="O9" s="13"/>
       <c r="Q9" s="7" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="R9" s="12"/>
       <c r="S9" s="12"/>
@@ -2958,36 +2866,36 @@
       </c>
       <c r="Q10" s="3"/>
       <c r="R10" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="Y10" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="AD10" s="2"/>
       <c r="AE10" s="2"/>
@@ -3038,37 +2946,37 @@
       <c r="O11" s="2"/>
       <c r="Q11" s="3"/>
       <c r="R11" s="3" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="W11" s="2" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="X11" s="2" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="Y11" s="3" t="s">
         <v>14</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="AA11" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="AB11" s="16" t="s">
-        <v>153</v>
+        <v>158</v>
+      </c>
+      <c r="AB11" s="17" t="s">
+        <v>159</v>
       </c>
       <c r="AC11" s="10" t="s">
         <v>93</v>
@@ -3120,37 +3028,37 @@
       <c r="O12" s="2"/>
       <c r="Q12" s="3"/>
       <c r="R12" s="3" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="X12" s="4" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="Y12" s="3" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="AB12" s="10" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="AC12" s="10" t="s">
         <v>94</v>
@@ -3202,37 +3110,37 @@
       <c r="O13" s="2"/>
       <c r="Q13" s="3"/>
       <c r="R13" s="3" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="U13" s="3" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="V13" s="3" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="Y13" s="3" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="Z13" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="AA13" s="3" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="AB13" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -3330,24 +3238,24 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
@@ -3363,10 +3271,10 @@
       <c r="M17" s="12"/>
       <c r="N17" s="12"/>
       <c r="O17" s="13"/>
-      <c r="Q17" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="R17" s="17"/>
+      <c r="Q17" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="R17" s="18"/>
       <c r="S17" s="12"/>
       <c r="T17" s="12"/>
       <c r="U17" s="12"/>
@@ -3383,7 +3291,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>109</v>
@@ -3491,7 +3399,7 @@
       <c r="X19" s="2"/>
       <c r="Y19" s="3"/>
       <c r="Z19" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="AA19" s="2"/>
       <c r="AB19" s="2"/>
@@ -3516,7 +3424,7 @@
         <v>85</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>87</v>
@@ -3548,14 +3456,14 @@
       <c r="U20" s="4"/>
       <c r="V20" s="2"/>
       <c r="W20" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="X20" s="4" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="Y20" s="3"/>
       <c r="Z20" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="AA20" s="2"/>
       <c r="AB20" s="2"/>
@@ -3589,7 +3497,7 @@
         <v>54</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="2"/>
@@ -3606,7 +3514,7 @@
       <c r="U21" s="2"/>
       <c r="V21" s="3"/>
       <c r="W21" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="X21" s="2"/>
       <c r="Y21" s="3"/>
@@ -3701,26 +3609,26 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="15"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+      <c r="O24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="B25" s="17"/>
+        <v>191</v>
+      </c>
+      <c r="B25" s="18"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12"/>
@@ -3737,10 +3645,10 @@
       <c r="P25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="Q25" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="R25" s="17"/>
+      <c r="Q25" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="R25" s="18"/>
       <c r="S25" s="12"/>
       <c r="T25" s="12"/>
       <c r="U25" s="12"/>
@@ -3859,13 +3767,13 @@
       <c r="V27" s="2"/>
       <c r="W27" s="2"/>
       <c r="X27" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="Y27" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="Z27" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="AA27" s="2"/>
       <c r="AB27" s="2"/>
@@ -3888,7 +3796,7 @@
         <v>85</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>87</v>
@@ -3922,16 +3830,16 @@
       <c r="U28" s="4"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="X28" s="4" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="Y28" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="Z28" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="AA28" s="2"/>
       <c r="AB28" s="2"/>
@@ -3965,7 +3873,7 @@
         <v>54</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="J29" s="3"/>
       <c r="K29" s="2"/>
@@ -3982,10 +3890,10 @@
       <c r="U29" s="2"/>
       <c r="V29" s="3"/>
       <c r="W29" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="X29" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="Y29" s="3"/>
       <c r="Z29" s="2"/>
@@ -4081,24 +3989,24 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="14"/>
-      <c r="K32" s="14"/>
-      <c r="L32" s="14"/>
-      <c r="M32" s="14"/>
-      <c r="N32" s="14"/>
-      <c r="O32" s="15"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
+      <c r="M32" s="15"/>
+      <c r="N32" s="15"/>
+      <c r="O32" s="16"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7"/>
-      <c r="B33" s="17"/>
+      <c r="B33" s="18"/>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
       <c r="E33" s="12"/>
@@ -4113,9 +4021,9 @@
       <c r="N33" s="12"/>
       <c r="O33" s="13"/>
       <c r="Q33" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="R33" s="17"/>
+        <v>195</v>
+      </c>
+      <c r="R33" s="18"/>
       <c r="S33" s="12"/>
       <c r="T33" s="12"/>
       <c r="U33" s="12"/>
@@ -4255,7 +4163,7 @@
       <c r="Q35" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="R35" s="19" t="s">
+      <c r="R35" s="20" t="s">
         <v>74</v>
       </c>
       <c r="S35" s="3" t="s">
@@ -4270,25 +4178,25 @@
       <c r="V35" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="W35" s="19" t="s">
+      <c r="W35" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="X35" s="19" t="s">
+      <c r="X35" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="Y35" s="19" t="s">
+      <c r="Y35" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="Z35" s="19" t="s">
+      <c r="Z35" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AA35" s="19" t="s">
+      <c r="AA35" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="AB35" s="19" t="s">
+      <c r="AB35" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="AC35" s="19" t="s">
+      <c r="AC35" s="20" t="s">
         <v>79</v>
       </c>
       <c r="AD35" s="2"/>
@@ -4309,7 +4217,7 @@
         <v>85</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>87</v>
@@ -4337,10 +4245,10 @@
       <c r="Q36" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="R36" s="19" t="s">
-        <v>190</v>
-      </c>
-      <c r="S36" s="19" t="s">
+      <c r="R36" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="S36" s="20" t="s">
         <v>83</v>
       </c>
       <c r="T36" s="3" t="s">
@@ -4349,28 +4257,28 @@
       <c r="U36" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="V36" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="W36" s="19" t="s">
+      <c r="V36" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="W36" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="X36" s="19" t="s">
+      <c r="X36" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="Y36" s="19" t="s">
+      <c r="Y36" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="Z36" s="19" t="s">
+      <c r="Z36" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="AA36" s="19" t="s">
+      <c r="AA36" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="AB36" s="19" t="s">
+      <c r="AB36" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="AC36" s="19" t="s">
+      <c r="AC36" s="20" t="s">
         <v>80</v>
       </c>
       <c r="AD36" s="2"/>
@@ -4402,10 +4310,10 @@
         <v>54</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
@@ -4420,22 +4328,22 @@
       <c r="R37" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="S37" s="19" t="s">
+      <c r="S37" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="T37" s="19" t="s">
+      <c r="T37" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="U37" s="19" t="s">
+      <c r="U37" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="V37" s="19" t="s">
+      <c r="V37" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="W37" s="19" t="s">
+      <c r="W37" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="X37" s="19" t="s">
+      <c r="X37" s="20" t="s">
         <v>54</v>
       </c>
       <c r="Y37" s="3"/>
@@ -4555,26 +4463,26 @@
       <c r="AE39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="18"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="14"/>
-      <c r="K40" s="14"/>
-      <c r="L40" s="14"/>
-      <c r="M40" s="14"/>
-      <c r="N40" s="14"/>
-      <c r="O40" s="15"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15"/>
+      <c r="L40" s="15"/>
+      <c r="M40" s="15"/>
+      <c r="N40" s="15"/>
+      <c r="O40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17" t="s">
-        <v>190</v>
-      </c>
-      <c r="B41" s="17"/>
+      <c r="A41" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="B41" s="18"/>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
       <c r="E41" s="12"/>
@@ -4588,10 +4496,10 @@
       <c r="M41" s="12"/>
       <c r="N41" s="12"/>
       <c r="O41" s="13"/>
-      <c r="Q41" s="17" t="s">
-        <v>192</v>
-      </c>
-      <c r="R41" s="17"/>
+      <c r="Q41" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="R41" s="18"/>
       <c r="S41" s="12"/>
       <c r="T41" s="12"/>
       <c r="U41" s="12"/>
@@ -4649,7 +4557,7 @@
       <c r="H43" s="2"/>
       <c r="I43" s="3"/>
       <c r="J43" s="2" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
@@ -4658,7 +4566,7 @@
       <c r="O43" s="2"/>
       <c r="Q43" s="3"/>
       <c r="R43" s="2" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
@@ -4666,14 +4574,14 @@
       <c r="V43" s="2"/>
       <c r="W43" s="2"/>
       <c r="X43" s="2" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="Y43" s="2" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="Z43" s="2"/>
       <c r="AA43" s="2" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="AB43" s="2"/>
       <c r="AC43" s="2"/>
@@ -4692,14 +4600,14 @@
       <c r="E44" s="4"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="I44" s="3"/>
       <c r="J44" s="2" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
@@ -4719,7 +4627,7 @@
       <c r="W44" s="2"/>
       <c r="X44" s="4"/>
       <c r="Y44" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="Z44" s="2"/>
       <c r="AA44" s="2"/>
@@ -4736,7 +4644,7 @@
       <c r="E45" s="2"/>
       <c r="F45" s="3"/>
       <c r="G45" s="2" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="H45" s="2"/>
       <c r="I45" s="3"/>
@@ -4758,15 +4666,15 @@
       </c>
       <c r="U45" s="3"/>
       <c r="V45" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="W45" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="X45" s="3"/>
       <c r="Y45" s="3"/>
       <c r="Z45" s="2"/>
-      <c r="AA45" s="20" t="s">
+      <c r="AA45" s="21" t="s">
         <v>43</v>
       </c>
       <c r="AB45" s="2"/>
@@ -4855,27 +4763,27 @@
       <c r="AE47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="18"/>
-      <c r="B48" s="18"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="14"/>
-      <c r="N48" s="14"/>
-      <c r="O48" s="15"/>
+      <c r="A48" s="19"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
+      <c r="M48" s="15"/>
+      <c r="N48" s="15"/>
+      <c r="O48" s="16"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="21" t="s">
-        <v>204</v>
-      </c>
-      <c r="B49" s="17"/>
+      <c r="A49" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="B49" s="18"/>
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
       <c r="E49" s="12"/>
@@ -4889,8 +4797,8 @@
       <c r="M49" s="12"/>
       <c r="N49" s="12"/>
       <c r="O49" s="13"/>
-      <c r="Q49" s="21" t="s">
-        <v>205</v>
+      <c r="Q49" s="7" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5024,7 +4932,7 @@
         <v>19</v>
       </c>
       <c r="AC51" s="2" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="AD51" s="2"/>
       <c r="AE51" s="2"/>
@@ -5032,37 +4940,37 @@
     <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>
       <c r="B52" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="M52" s="10" t="s">
         <v>94</v>
@@ -5088,13 +4996,13 @@
         <v>3</v>
       </c>
       <c r="AA52" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="AB52" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="AC52" s="2" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="AD52" s="2"/>
       <c r="AE52" s="2"/>
@@ -5119,22 +5027,22 @@
         <v>81</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>2</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="K53" s="3" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="L53" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="M53" s="2" t="s">
         <v>33</v>
@@ -5185,10 +5093,10 @@
         <v>49</v>
       </c>
       <c r="G54" s="3"/>
-      <c r="H54" s="20" t="s">
+      <c r="H54" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="I54" s="20" t="s">
+      <c r="I54" s="21" t="s">
         <v>58</v>
       </c>
       <c r="J54" s="6"/>
@@ -5223,8 +5131,8 @@
       <c r="E55" s="8"/>
       <c r="F55" s="8"/>
       <c r="G55" s="3"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
+      <c r="H55" s="21"/>
+      <c r="I55" s="21"/>
       <c r="J55" s="6"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
@@ -5840,24 +5748,24 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -6114,24 +6022,24 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
@@ -6288,7 +6196,7 @@
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="M21" s="2" t="s">
         <v>33</v>
@@ -6355,26 +6263,26 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="15"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15"/>
+      <c r="M24" s="15"/>
+      <c r="N24" s="15"/>
+      <c r="O24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="B25" s="17"/>
+        <v>191</v>
+      </c>
+      <c r="B25" s="18"/>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
       <c r="E25" s="12"/>
@@ -6436,13 +6344,13 @@
       <c r="F27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="H27" s="19" t="s">
+      <c r="H27" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="I27" s="19" t="s">
+      <c r="I27" s="20" t="s">
         <v>52</v>
       </c>
       <c r="J27" s="2" t="s">
@@ -6460,34 +6368,34 @@
     </row>
     <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3"/>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="D28" s="19" t="s">
+      <c r="D28" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="E28" s="19" t="s">
+      <c r="E28" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="F28" s="19" t="s">
+      <c r="F28" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="G28" s="19" t="s">
+      <c r="G28" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="H28" s="19" t="s">
+      <c r="H28" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="I28" s="19" t="s">
+      <c r="I28" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="J28" s="19" t="s">
+      <c r="J28" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="K28" s="19" t="s">
+      <c r="K28" s="20" t="s">
         <v>19</v>
       </c>
       <c r="L28" s="2"/>
@@ -6502,19 +6410,19 @@
       <c r="B29" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C29" s="19" t="s">
+      <c r="C29" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D29" s="19" t="s">
+      <c r="D29" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="E29" s="19" t="s">
+      <c r="E29" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="20" t="s">
         <v>92</v>
       </c>
       <c r="H29" s="22" t="s">
@@ -6528,7 +6436,7 @@
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="M29" s="2" t="s">
         <v>33</v>
@@ -6588,26 +6496,26 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="14"/>
-      <c r="J32" s="14"/>
-      <c r="K32" s="14"/>
-      <c r="L32" s="14"/>
-      <c r="M32" s="14"/>
-      <c r="N32" s="14"/>
-      <c r="O32" s="15"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
+      <c r="M32" s="15"/>
+      <c r="N32" s="15"/>
+      <c r="O32" s="16"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="B33" s="17"/>
+        <v>212</v>
+      </c>
+      <c r="B33" s="18"/>
       <c r="C33" s="12"/>
       <c r="D33" s="12"/>
       <c r="E33" s="12"/>
@@ -6707,37 +6615,37 @@
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="M36" s="10" t="s">
         <v>94</v>
@@ -6783,7 +6691,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>18</v>
@@ -6804,16 +6712,16 @@
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>33</v>
@@ -6874,10 +6782,10 @@
         <v>49</v>
       </c>
       <c r="G38" s="3"/>
-      <c r="H38" s="20" t="s">
+      <c r="H38" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="I38" s="20" t="s">
+      <c r="I38" s="21" t="s">
         <v>58</v>
       </c>
       <c r="J38" s="6"/>
@@ -6897,8 +6805,8 @@
       <c r="E39" s="8"/>
       <c r="F39" s="8"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="21"/>
       <c r="J39" s="6"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
@@ -6907,26 +6815,26 @@
       <c r="O39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="18"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="14"/>
-      <c r="K40" s="14"/>
-      <c r="L40" s="14"/>
-      <c r="M40" s="14"/>
-      <c r="N40" s="14"/>
-      <c r="O40" s="15"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15"/>
+      <c r="K40" s="15"/>
+      <c r="L40" s="15"/>
+      <c r="M40" s="15"/>
+      <c r="N40" s="15"/>
+      <c r="O40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="B41" s="17"/>
+        <v>213</v>
+      </c>
+      <c r="B41" s="18"/>
       <c r="C41" s="12"/>
       <c r="D41" s="12"/>
       <c r="E41" s="12"/>
@@ -7134,27 +7042,27 @@
       <c r="O47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="18"/>
-      <c r="B48" s="18"/>
-      <c r="C48" s="14"/>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="14"/>
-      <c r="N48" s="14"/>
-      <c r="O48" s="15"/>
+      <c r="A48" s="19"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
+      <c r="I48" s="15"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
+      <c r="M48" s="15"/>
+      <c r="N48" s="15"/>
+      <c r="O48" s="16"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="B49" s="17"/>
+      <c r="A49" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="B49" s="18"/>
       <c r="C49" s="12"/>
       <c r="D49" s="12"/>
       <c r="E49" s="12"/>
@@ -7213,14 +7121,14 @@
       <c r="E52" s="4"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
@@ -7236,7 +7144,7 @@
       <c r="E53" s="2"/>
       <c r="F53" s="3"/>
       <c r="G53" s="2" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="H53" s="2"/>
       <c r="I53" s="3"/>

</xml_diff>

<commit_message>
[Update] Operation of mouse mode has been changed.
</commit_message>
<xml_diff>
--- a/misc/keymap.xlsx
+++ b/misc/keymap.xlsx
@@ -8,9 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="space modifier" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="space modifier_2" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="space modifier_2_2" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="space modifier" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="space modifier_2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="space modifier_2_2" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1159" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1155" uniqueCount="217">
   <si>
     <t xml:space="preserve">標準</t>
   </si>
@@ -429,6 +429,9 @@
     <t xml:space="preserve">右クリック</t>
   </si>
   <si>
+    <t xml:space="preserve">Norml</t>
+  </si>
+  <si>
     <t xml:space="preserve">WhlUp</t>
   </si>
   <si>
@@ -438,6 +441,12 @@
     <t xml:space="preserve">Back</t>
   </si>
   <si>
+    <t xml:space="preserve">Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Next</t>
+  </si>
+  <si>
     <t xml:space="preserve">標準(レジストリ編集)</t>
   </si>
   <si>
@@ -573,9 +582,6 @@
     <t xml:space="preserve">F13修飾</t>
   </si>
   <si>
-    <t xml:space="preserve">無変換 修飾</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reload</t>
   </si>
   <si>
@@ -594,6 +600,9 @@
     <t xml:space="preserve">Num</t>
   </si>
   <si>
+    <t xml:space="preserve">Mouse</t>
+  </si>
+  <si>
     <t xml:space="preserve">S+End</t>
   </si>
   <si>
@@ -615,9 +624,6 @@
     <t xml:space="preserve">Space &amp; F13 修飾</t>
   </si>
   <si>
-    <t xml:space="preserve">APP</t>
-  </si>
-  <si>
     <t xml:space="preserve">/ 修飾   C+k,C+{}</t>
   </si>
   <si>
@@ -657,7 +663,7 @@
     <t xml:space="preserve"> (F14 or 変換 or 無変換) 修飾</t>
   </si>
   <si>
-    <t xml:space="preserve">Lock</t>
+    <t xml:space="preserve">Layer1</t>
   </si>
   <si>
     <t xml:space="preserve">ひらがな./変換/無変換　修飾</t>
@@ -1058,6 +1064,112 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -2535,8 +2647,8 @@
       <c r="X3" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="Y3" s="3" t="n">
-        <v>5</v>
+      <c r="Y3" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="Z3" s="14" t="s">
         <v>134</v>
@@ -2589,14 +2701,16 @@
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
-      <c r="Q4" s="3"/>
+      <c r="Q4" s="3" t="s">
+        <v>135</v>
+      </c>
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="4"/>
       <c r="V4" s="2"/>
       <c r="W4" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="X4" s="4" t="s">
         <v>53</v>
@@ -2662,10 +2776,10 @@
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
       <c r="W5" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
@@ -2716,14 +2830,18 @@
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
+      <c r="V6" s="3" t="s">
+        <v>139</v>
+      </c>
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
       <c r="Y6" s="3"/>
       <c r="Z6" s="6"/>
       <c r="AA6" s="2"/>
       <c r="AB6" s="6"/>
-      <c r="AC6" s="2"/>
+      <c r="AC6" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="AD6" s="6"/>
       <c r="AE6" s="6"/>
     </row>
@@ -2760,9 +2878,15 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="6"/>
       <c r="AA7" s="2"/>
-      <c r="AB7" s="2"/>
-      <c r="AC7" s="2"/>
-      <c r="AD7" s="2"/>
+      <c r="AB7" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="AC7" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="AD7" s="2" t="s">
+        <v>140</v>
+      </c>
       <c r="AE7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2784,7 +2908,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2801,7 +2925,7 @@
       <c r="N9" s="12"/>
       <c r="O9" s="13"/>
       <c r="Q9" s="7" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="R9" s="12"/>
       <c r="S9" s="12"/>
@@ -2866,36 +2990,36 @@
       </c>
       <c r="Q10" s="3"/>
       <c r="R10" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="Y10" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
       <c r="AC10" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="AD10" s="2"/>
       <c r="AE10" s="2"/>
@@ -2946,37 +3070,37 @@
       <c r="O11" s="2"/>
       <c r="Q11" s="3"/>
       <c r="R11" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="W11" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="X11" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="Y11" s="3" t="s">
         <v>14</v>
       </c>
       <c r="Z11" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AA11" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="AB11" s="17" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="AC11" s="10" t="s">
         <v>93</v>
@@ -3028,37 +3152,37 @@
       <c r="O12" s="2"/>
       <c r="Q12" s="3"/>
       <c r="R12" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="U12" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="W12" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="X12" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="Y12" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="Z12" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="AA12" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AB12" s="10" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AC12" s="10" t="s">
         <v>94</v>
@@ -3110,37 +3234,37 @@
       <c r="O13" s="2"/>
       <c r="Q13" s="3"/>
       <c r="R13" s="3" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="U13" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="V13" s="3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="Y13" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="Z13" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AA13" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="AB13" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
@@ -3255,7 +3379,7 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
@@ -3271,9 +3395,7 @@
       <c r="M17" s="12"/>
       <c r="N17" s="12"/>
       <c r="O17" s="13"/>
-      <c r="Q17" s="18" t="s">
-        <v>183</v>
-      </c>
+      <c r="Q17" s="18"/>
       <c r="R17" s="18"/>
       <c r="S17" s="12"/>
       <c r="T17" s="12"/>
@@ -3291,7 +3413,7 @@
     </row>
     <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>109</v>
@@ -3399,7 +3521,7 @@
       <c r="X19" s="2"/>
       <c r="Y19" s="3"/>
       <c r="Z19" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AA19" s="2"/>
       <c r="AB19" s="2"/>
@@ -3424,7 +3546,7 @@
         <v>85</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>87</v>
@@ -3456,14 +3578,14 @@
       <c r="U20" s="4"/>
       <c r="V20" s="2"/>
       <c r="W20" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="X20" s="4" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="Y20" s="3"/>
       <c r="Z20" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AA20" s="2"/>
       <c r="AB20" s="2"/>
@@ -3497,9 +3619,11 @@
         <v>54</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="J21" s="3"/>
+        <v>191</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>192</v>
+      </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2" t="s">
@@ -3514,7 +3638,7 @@
       <c r="U21" s="2"/>
       <c r="V21" s="3"/>
       <c r="W21" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="X21" s="2"/>
       <c r="Y21" s="3"/>
@@ -3626,7 +3750,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="12"/>
@@ -3646,7 +3770,7 @@
         <v>42</v>
       </c>
       <c r="Q25" s="18" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="R25" s="18"/>
       <c r="S25" s="12"/>
@@ -3767,13 +3891,13 @@
       <c r="V27" s="2"/>
       <c r="W27" s="2"/>
       <c r="X27" s="3" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="Y27" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="Z27" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AA27" s="2"/>
       <c r="AB27" s="2"/>
@@ -3796,7 +3920,7 @@
         <v>85</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>87</v>
@@ -3830,16 +3954,16 @@
       <c r="U28" s="4"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="X28" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="Y28" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="Z28" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="X28" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="Y28" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="Z28" s="2" t="s">
-        <v>185</v>
       </c>
       <c r="AA28" s="2"/>
       <c r="AB28" s="2"/>
@@ -3873,9 +3997,11 @@
         <v>54</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="J29" s="3"/>
+        <v>191</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>192</v>
+      </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2" t="s">
@@ -3890,10 +4016,10 @@
       <c r="U29" s="2"/>
       <c r="V29" s="3"/>
       <c r="W29" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="X29" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="Y29" s="3"/>
       <c r="Z29" s="2"/>
@@ -4021,7 +4147,7 @@
       <c r="N33" s="12"/>
       <c r="O33" s="13"/>
       <c r="Q33" s="7" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="R33" s="18"/>
       <c r="S33" s="12"/>
@@ -4217,7 +4343,7 @@
         <v>85</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>87</v>
@@ -4246,7 +4372,7 @@
         <v>57</v>
       </c>
       <c r="R36" s="20" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="S36" s="20" t="s">
         <v>83</v>
@@ -4258,7 +4384,7 @@
         <v>85</v>
       </c>
       <c r="V36" s="20" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="W36" s="20" t="s">
         <v>87</v>
@@ -4309,12 +4435,8 @@
       <c r="H37" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="I37" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>197</v>
-      </c>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
       <c r="M37" s="2" t="s">
@@ -4370,9 +4492,7 @@
         <v>47</v>
       </c>
       <c r="E38" s="3"/>
-      <c r="F38" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="2" t="s">
         <v>1</v>
@@ -4480,7 +4600,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="18" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B41" s="18"/>
       <c r="C41" s="12"/>
@@ -4497,7 +4617,7 @@
       <c r="N41" s="12"/>
       <c r="O41" s="13"/>
       <c r="Q41" s="18" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="R41" s="18"/>
       <c r="S41" s="12"/>
@@ -4557,7 +4677,7 @@
       <c r="H43" s="2"/>
       <c r="I43" s="3"/>
       <c r="J43" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
@@ -4566,7 +4686,7 @@
       <c r="O43" s="2"/>
       <c r="Q43" s="3"/>
       <c r="R43" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
@@ -4574,20 +4694,18 @@
       <c r="V43" s="2"/>
       <c r="W43" s="2"/>
       <c r="X43" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="Y43" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="Z43" s="2"/>
       <c r="AA43" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="AB43" s="2"/>
       <c r="AC43" s="2"/>
-      <c r="AD43" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="AD43" s="2"/>
       <c r="AE43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4600,14 +4718,14 @@
       <c r="E44" s="4"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I44" s="3"/>
       <c r="J44" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="K44" s="2"/>
       <c r="L44" s="2"/>
@@ -4627,7 +4745,7 @@
       <c r="W44" s="2"/>
       <c r="X44" s="4"/>
       <c r="Y44" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="Z44" s="2"/>
       <c r="AA44" s="2"/>
@@ -4644,7 +4762,7 @@
       <c r="E45" s="2"/>
       <c r="F45" s="3"/>
       <c r="G45" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H45" s="2"/>
       <c r="I45" s="3"/>
@@ -4654,9 +4772,7 @@
       <c r="M45" s="2"/>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
-      <c r="Q45" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="Q45" s="3"/>
       <c r="R45" s="3"/>
       <c r="S45" s="3" t="s">
         <v>89</v>
@@ -4666,10 +4782,10 @@
       </c>
       <c r="U45" s="3"/>
       <c r="V45" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="W45" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="X45" s="3"/>
       <c r="Y45" s="3"/>
@@ -4678,9 +4794,7 @@
         <v>43</v>
       </c>
       <c r="AB45" s="2"/>
-      <c r="AC45" s="2" t="s">
-        <v>33</v>
-      </c>
+      <c r="AC45" s="2"/>
       <c r="AD45" s="2"/>
       <c r="AE45" s="2"/>
     </row>
@@ -4702,29 +4816,17 @@
       <c r="M46" s="2"/>
       <c r="N46" s="6"/>
       <c r="O46" s="6"/>
-      <c r="Q46" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="R46" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="S46" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="T46" s="3" t="s">
-        <v>47</v>
-      </c>
+      <c r="Q46" s="3"/>
+      <c r="R46" s="3"/>
+      <c r="S46" s="3"/>
+      <c r="T46" s="3"/>
       <c r="U46" s="3"/>
-      <c r="V46" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="V46" s="3"/>
       <c r="W46" s="3"/>
       <c r="X46" s="2"/>
       <c r="Y46" s="3"/>
       <c r="Z46" s="6"/>
-      <c r="AA46" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="AA46" s="2"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="2"/>
       <c r="AD46" s="6"/>
@@ -4781,7 +4883,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B49" s="18"/>
       <c r="C49" s="12"/>
@@ -4798,7 +4900,7 @@
       <c r="N49" s="12"/>
       <c r="O49" s="13"/>
       <c r="Q49" s="7" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4932,7 +5034,7 @@
         <v>19</v>
       </c>
       <c r="AC51" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="AD51" s="2"/>
       <c r="AE51" s="2"/>
@@ -4940,44 +5042,46 @@
     <row r="52" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>
       <c r="B52" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="M52" s="10" t="s">
         <v>94</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
-      <c r="Q52" s="3"/>
+      <c r="Q52" s="3" t="s">
+        <v>139</v>
+      </c>
       <c r="R52" s="3"/>
       <c r="S52" s="3"/>
       <c r="T52" s="3"/>
@@ -4996,13 +5100,13 @@
         <v>3</v>
       </c>
       <c r="AA52" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AB52" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AC52" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="AD52" s="2"/>
       <c r="AE52" s="2"/>
@@ -5027,22 +5131,22 @@
         <v>81</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>2</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K53" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="L53" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="M53" s="2" t="s">
         <v>33</v>
@@ -5077,9 +5181,7 @@
       <c r="A54" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B54" s="3" t="s">
-        <v>45</v>
-      </c>
+      <c r="B54" s="3"/>
       <c r="C54" s="3" t="s">
         <v>46</v>
       </c>
@@ -5089,9 +5191,7 @@
       <c r="E54" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F54" s="3" t="s">
-        <v>49</v>
-      </c>
+      <c r="F54" s="3"/>
       <c r="G54" s="3"/>
       <c r="H54" s="21" t="s">
         <v>50</v>
@@ -5112,7 +5212,9 @@
       <c r="S54" s="3"/>
       <c r="T54" s="3"/>
       <c r="U54" s="3"/>
-      <c r="V54" s="3"/>
+      <c r="V54" s="3" t="s">
+        <v>139</v>
+      </c>
       <c r="W54" s="3"/>
       <c r="X54" s="3"/>
       <c r="Y54" s="3"/>
@@ -5765,7 +5867,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -6039,7 +6141,7 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
@@ -6196,7 +6298,7 @@
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="M21" s="2" t="s">
         <v>33</v>
@@ -6280,7 +6382,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B25" s="18"/>
       <c r="C25" s="12"/>
@@ -6436,7 +6538,7 @@
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="M29" s="2" t="s">
         <v>33</v>
@@ -6513,7 +6615,7 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B33" s="18"/>
       <c r="C33" s="12"/>
@@ -6615,37 +6717,37 @@
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="L36" s="10" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="M36" s="10" t="s">
         <v>94</v>
@@ -6691,7 +6793,7 @@
         <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>18</v>
@@ -6712,16 +6814,16 @@
         <v>2</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="M37" s="2" t="s">
         <v>33</v>
@@ -6832,7 +6934,7 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B41" s="18"/>
       <c r="C41" s="12"/>
@@ -7060,7 +7162,7 @@
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B49" s="18"/>
       <c r="C49" s="12"/>
@@ -7121,14 +7223,14 @@
       <c r="E52" s="4"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="2"/>
@@ -7144,7 +7246,7 @@
       <c r="E53" s="2"/>
       <c r="F53" s="3"/>
       <c r="G53" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H53" s="2"/>
       <c r="I53" s="3"/>

</xml_diff>